<commit_message>
update profile descr 2a8b02f66585a55db43a67538f9f6d5a3e0005d3
</commit_message>
<xml_diff>
--- a/nr-add-examples/ig/StructureDefinition-pdsm-find-documentreferences-comprehensive-response.xlsx
+++ b/nr-add-examples/ig/StructureDefinition-pdsm-find-documentreferences-comprehensive-response.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-04-30T08:28:31+00:00</t>
+    <t>2025-04-30T11:32:46+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -81,7 +81,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Profil de réponse de la transaction IHE "Find Document References [ITI-67]" basée sur le bundle MHD FindDocumentReferencesComprehensiveResponseMessage et profilé pour le volet PDSm</t>
+    <t>Profil de réponse de la transaction IHE "Find Document References [ITI-67]" basée sur le bundle MHD FindDocumentReferencesComprehensiveResponseMessage</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>